<commit_message>
added more functionality 711-626
</commit_message>
<xml_diff>
--- a/docs/Manual_Test_Plan.xlsx
+++ b/docs/Manual_Test_Plan.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/sharad/techWork/Baseball/dsa_wp_modern_prototype/docs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:9_{FB652D03-FC0C-2249-B081-0D05EC704DA0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:9_{F223A772-321B-4948-9EB6-4065CBFC7F10}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="34600" yWindow="720" windowWidth="34160" windowHeight="25520" xr2:uid="{12D105A3-D4DE-D04D-A0F5-AABFBDED4B2E}"/>
   </bookViews>
@@ -3167,10 +3167,10 @@
         <v>54</v>
       </c>
       <c r="G10" s="5" t="s">
-        <v>626</v>
+        <v>625</v>
       </c>
       <c r="H10" s="6" t="s">
-        <v>626</v>
+        <v>627</v>
       </c>
       <c r="I10" s="4"/>
     </row>
@@ -3194,10 +3194,10 @@
         <v>59</v>
       </c>
       <c r="G11" s="5" t="s">
-        <v>626</v>
+        <v>625</v>
       </c>
       <c r="H11" s="6" t="s">
-        <v>626</v>
+        <v>627</v>
       </c>
       <c r="I11" s="4"/>
     </row>
@@ -3221,10 +3221,10 @@
         <v>64</v>
       </c>
       <c r="G12" s="5" t="s">
-        <v>626</v>
+        <v>625</v>
       </c>
       <c r="H12" s="6" t="s">
-        <v>626</v>
+        <v>627</v>
       </c>
       <c r="I12" s="4"/>
     </row>
@@ -3248,10 +3248,10 @@
         <v>69</v>
       </c>
       <c r="G13" s="5" t="s">
-        <v>626</v>
+        <v>625</v>
       </c>
       <c r="H13" s="6" t="s">
-        <v>626</v>
+        <v>627</v>
       </c>
       <c r="I13" s="4"/>
     </row>
@@ -3275,10 +3275,10 @@
         <v>74</v>
       </c>
       <c r="G14" s="5" t="s">
-        <v>626</v>
+        <v>625</v>
       </c>
       <c r="H14" s="6" t="s">
-        <v>626</v>
+        <v>627</v>
       </c>
       <c r="I14" s="4"/>
     </row>
@@ -3302,10 +3302,10 @@
         <v>79</v>
       </c>
       <c r="G15" s="5" t="s">
-        <v>626</v>
+        <v>625</v>
       </c>
       <c r="H15" s="6" t="s">
-        <v>626</v>
+        <v>627</v>
       </c>
       <c r="I15" s="4"/>
     </row>
@@ -3329,10 +3329,10 @@
         <v>84</v>
       </c>
       <c r="G16" s="5" t="s">
-        <v>626</v>
+        <v>625</v>
       </c>
       <c r="H16" s="6" t="s">
-        <v>626</v>
+        <v>627</v>
       </c>
       <c r="I16" s="4"/>
     </row>
@@ -3356,10 +3356,10 @@
         <v>89</v>
       </c>
       <c r="G17" s="5" t="s">
-        <v>626</v>
+        <v>625</v>
       </c>
       <c r="H17" s="6" t="s">
-        <v>626</v>
+        <v>627</v>
       </c>
       <c r="I17" s="4"/>
     </row>
@@ -3383,10 +3383,10 @@
         <v>94</v>
       </c>
       <c r="G18" s="5" t="s">
-        <v>626</v>
+        <v>625</v>
       </c>
       <c r="H18" s="6" t="s">
-        <v>626</v>
+        <v>627</v>
       </c>
       <c r="I18" s="4"/>
     </row>
@@ -3410,10 +3410,10 @@
         <v>99</v>
       </c>
       <c r="G19" s="5" t="s">
-        <v>626</v>
+        <v>625</v>
       </c>
       <c r="H19" s="6" t="s">
-        <v>626</v>
+        <v>627</v>
       </c>
       <c r="I19" s="4"/>
     </row>
@@ -3437,10 +3437,10 @@
         <v>104</v>
       </c>
       <c r="G20" s="5" t="s">
-        <v>626</v>
+        <v>625</v>
       </c>
       <c r="H20" s="6" t="s">
-        <v>626</v>
+        <v>627</v>
       </c>
       <c r="I20" s="4"/>
     </row>
@@ -3464,10 +3464,10 @@
         <v>109</v>
       </c>
       <c r="G21" s="5" t="s">
-        <v>626</v>
+        <v>625</v>
       </c>
       <c r="H21" s="6" t="s">
-        <v>626</v>
+        <v>627</v>
       </c>
       <c r="I21" s="4"/>
     </row>

</xml_diff>